<commit_message>
Fix scan reliability and add finding evidence
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/backend-tests/reports/endpoint-inventory.xlsx
+++ b/backend-tests/reports/endpoint-inventory.xlsx
@@ -794,7 +794,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Bearer (NO ownership check -- VULN-001)</t>
+          <t>Authenticated; client access is scan-owner scoped</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -816,12 +816,12 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Bearer (analyst/admin)</t>
+          <t>Authenticated; client access is scan-owner scoped</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Update triage status</t>
+          <t>Fetch one vulnerability</t>
         </is>
       </c>
     </row>
@@ -838,7 +838,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Bearer (NO ownership/role check -- VULN-006)</t>
+          <t>Authenticated; client access is scan-owner scoped</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Bearer (NOT tenant-scoped -- VULN-001)</t>
+          <t>Authenticated; client results are tenant-scoped</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Bearer (NO ownership check -- VULN-001)</t>
+          <t>Authenticated; client access is scan-owner scoped</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Bearer (NO role check -- VULN-006)</t>
+          <t>Analyst/admin only; remediation must be APPROVED</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -992,12 +992,12 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Bearer (admin)</t>
+          <t>Admin only</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>List system config (hardcoded -- VULN-010)</t>
+          <t>List persisted runtime configuration</t>
         </is>
       </c>
     </row>
@@ -1014,12 +1014,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Bearer (admin)</t>
+          <t>Admin only</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Update config (NOT persisted -- VULN-010)</t>
+          <t>Update persisted runtime configuration</t>
         </is>
       </c>
     </row>
@@ -1058,12 +1058,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Bearer (admin)</t>
+          <t>Admin only</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Trigger NVD CVE sync</t>
+          <t>Manual NVD sync is unavailable; endpoint returns 501</t>
         </is>
       </c>
     </row>

</xml_diff>